<commit_message>
Add direct bird image links and configure overlay display in explorer profile
</commit_message>
<xml_diff>
--- a/Location/species_master.xlsx
+++ b/Location/species_master.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I130"/>
+  <dimension ref="A1:J130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,6 +474,11 @@
           <t>indicator group</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>image link</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -516,9 +521,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/b/bc/Ashy_drongo_in_Latpanchar_April_2024_by_Tisha_Mukherjee_01.jpg</t>
         </is>
       </c>
     </row>
@@ -563,9 +569,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/d/d1/Ashy_Prinia_in_Ajodhya_Hills_July_2024_by_Tisha_Mukherjee_01.jpg</t>
         </is>
       </c>
     </row>
@@ -610,9 +617,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/7/73/Av_Ashy_Woodswallow_THAI_JG.jpg</t>
         </is>
       </c>
     </row>
@@ -657,9 +665,10 @@
           <t>Arboreal (lower to midstory)</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/5/5b/Asian_brown_flycatcher_%28Muscicapa_dauurica_siamensis%29_Angkor_2.jpg/3840px-Asian_brown_flycatcher_%28Muscicapa_dauurica_siamensis%29_Angkor_2.jpg</t>
         </is>
       </c>
     </row>
@@ -709,6 +718,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/7/7e/Asian_Emerald_Dove_0A2A7379.jpg/3840px-Asian_Emerald_Dove_0A2A7379.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -751,9 +765,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/4/4a/Asian_koel.jpg</t>
         </is>
       </c>
     </row>
@@ -798,9 +813,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/f/fd/Asian_Palm_Swift_Cypsiurus_balasiensis_in_flight_02.JPG</t>
         </is>
       </c>
     </row>
@@ -845,9 +861,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/a/a8/Sand_martin_%28Riparia_riparia%29%2C_Guidel-Plage%2C_Brittany%2C_France_%2819765483180%29.jpg</t>
         </is>
       </c>
     </row>
@@ -892,9 +909,10 @@
           <t>Aerial / low arboreal interface</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/f/f9/Bdrongo-Sandeep1.jpg</t>
         </is>
       </c>
     </row>
@@ -939,9 +957,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/a/a1/Nycticorax_nycticorax_457953189.jpg</t>
         </is>
       </c>
     </row>
@@ -986,9 +1005,10 @@
           <t>Arboreal (midstory to canopy specialist)</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/a/a5/Cuckooshrike-blackheaded.jpg</t>
         </is>
       </c>
     </row>
@@ -1033,9 +1053,10 @@
           <t>Arboreal (midstory to canopy)</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/e/ec/Black-hooded_Oriole_in_Rabindra_Sarobar_January_2025_by_Tisha_Mukherjee_01.jpg/3840px-Black-hooded_Oriole_in_Rabindra_Sarobar_January_2025_by_Tisha_Mukherjee_01.jpg</t>
         </is>
       </c>
     </row>
@@ -1085,6 +1106,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/a/a6/Hypothymis_azurea_-_Kaeng_Krachan.jpg/3840px-Hypothymis_azurea_-_Kaeng_Krachan.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1127,9 +1153,10 @@
           <t>Arboreal (trunk specialist)</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/a/a5/BR-FlamebackM-Sandeep.jpg</t>
         </is>
       </c>
     </row>
@@ -1174,9 +1201,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/b/b2/Blue-tailed_Bee-eater_in_Sundarbans_National_Park_July_2025_by_Tisha_Mukherjee_03.jpg</t>
         </is>
       </c>
     </row>
@@ -1226,6 +1254,11 @@
           <t>Lantana-associated</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/f/fc/Blyth%27s_Reed_Warbler_in_Baruipur_December_2024_by_Tisha_Mukherjee_02.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1268,9 +1301,10 @@
           <t>Arboreal (low to midstory) with occasional ground use</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/8/8b/Brahminy_starling_-_Vadodara_2021-06-22.jpg</t>
         </is>
       </c>
     </row>
@@ -1320,6 +1354,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/4/4c/Bronzed-Drongo-Sandeep.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1362,9 +1401,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/6/64/Lanius_cristatus_-_Surin.jpg</t>
         </is>
       </c>
     </row>
@@ -1414,6 +1454,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/b/b7/Brown-breasted_flycatcher_%28Muscicapa_muttui%29.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1461,6 +1506,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/c/cb/Alcippe_poioicephala_davisoni_-_Kaeng_Krachan.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1508,6 +1558,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/b/b7/Changeable_Hawk_Eagle_Bandipur.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1550,9 +1605,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/f/fc/Chestnut-headed_bee-eater_%28Merops_leschenaulti%29_Yala.jpg</t>
         </is>
       </c>
     </row>
@@ -1597,9 +1653,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/b/b8/Cinereous_tit_%28Parus_cinereus%29_Photograph_by_Shantanu_Kuveskar.jpg</t>
         </is>
       </c>
     </row>
@@ -1644,9 +1701,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/8/85/Common_Chiffchaff_2025_04_04_01.jpg/3840px-Common_Chiffchaff_2025_04_04_01.jpg</t>
         </is>
       </c>
     </row>
@@ -1691,9 +1749,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/f/fd/Common_crane_grus_grus.jpg</t>
         </is>
       </c>
     </row>
@@ -1738,9 +1797,10 @@
           <t>Ground/water feeder</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/c/c5/Common-Greenshank.jpg</t>
         </is>
       </c>
     </row>
@@ -1785,9 +1845,10 @@
           <t>Arboreal (midstory to canopy)</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/9/9d/Cuculus_varius_India.jpg</t>
         </is>
       </c>
     </row>
@@ -1832,9 +1893,10 @@
           <t>Arboreal (lower to midstory)</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/8/87/Common-ioraM-Sandeep.jpg</t>
         </is>
       </c>
     </row>
@@ -1879,9 +1941,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/b/bc/Alcedo_atthis_-England-8_%28cropped%29.jpg</t>
         </is>
       </c>
     </row>
@@ -1926,9 +1989,10 @@
           <t>Primarily ground-feeding with arboreal use</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/3/3c/Acridotheres_tristis00.jpg</t>
         </is>
       </c>
     </row>
@@ -1973,9 +2037,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/1/19/Carpodacus_erythrinus_284921386.jpg</t>
         </is>
       </c>
     </row>
@@ -2020,9 +2085,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/a/a7/Actitis_hypoleucos_-_Laem_Pak_Bia.jpg</t>
         </is>
       </c>
     </row>
@@ -2067,9 +2133,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/c/c6/Common_snipe_%28Gallinago_gallinago%29_2022.jpg/3840px-Common_snipe_%28Gallinago_gallinago%29_2022.jpg</t>
         </is>
       </c>
     </row>
@@ -2119,6 +2186,11 @@
           <t>Lantana-associated</t>
         </is>
       </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/9/93/Common_tailorbird_%28Orthotomus_sutorius%29.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2161,9 +2233,10 @@
           <t>Arboreal (midstory to canopy)</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/5/5f/Common_Woodshrike_%28Tephrodornis_pondicerianus%29_Photograph_By_Shantanu_Kuveskar.jpg</t>
         </is>
       </c>
     </row>
@@ -2208,9 +2281,10 @@
           <t>Arboreal</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/f/fd/Coppersmith_Barbet_%28Megalaima_haemacephala%29_by_Shantanu_Kuveskar.jpg</t>
         </is>
       </c>
     </row>
@@ -2260,6 +2334,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/3/37/Spilornis_cheela_%28Bandipur%2C_2008%29.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2307,6 +2386,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/2/2f/Crimson-backed_sunbird_or_small_sunbird_%28Leptocoma_minima%29_by_Shantanu_Kuveskar.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2349,9 +2433,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/3/39/Dunlin_%28Calidris_alpina%29_in_the_Delaware_Bay_at_Heislerville_Wildlife_Management_Area%2C_New_Jersey%2C_USA.png</t>
         </is>
       </c>
     </row>
@@ -2396,9 +2481,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/d/d9/Eurasian_Coot_2023_11_25_03.jpg/3840px-Eurasian_Coot_2023_11_25_03.jpg</t>
         </is>
       </c>
     </row>
@@ -2443,9 +2529,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/2/2c/Eurasian_Curlew.jpg</t>
         </is>
       </c>
     </row>
@@ -2490,9 +2577,10 @@
           <t>Ground-feeding (terrestrial specialist)</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/6/62/Israel._Eurasian_Hoopoe_%286497645007%29.jpg/3840px-Israel._Eurasian_Hoopoe_%286497645007%29.jpg</t>
         </is>
       </c>
     </row>
@@ -2537,9 +2625,10 @@
           <t>Aquatic/ground interface</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/e/ee/Common_moorhen_%28Gallinula_chloropus%29_France.jpg/3840px-Common_moorhen_%28Gallinula_chloropus%29_France.jpg</t>
         </is>
       </c>
     </row>
@@ -2589,6 +2678,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/1/1f/Flame-throated_bulbul.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2631,9 +2725,10 @@
           <t>Arboreal (midstory to canopy specialist)</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/1/1b/Golden_Fronted_Leafbird_Mukulhinge.jpg</t>
         </is>
       </c>
     </row>
@@ -2678,9 +2773,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/f/f9/Grey_Francolin_in_Bhigwan_August_2025_by_Tisha_Mukherjee_04.jpg/3840px-Grey_Francolin_in_Bhigwan_August_2025_by_Tisha_Mukherjee_04.jpg</t>
         </is>
       </c>
     </row>
@@ -2725,9 +2821,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/7/71/Grey_heron_2022_03_18_01.jpg/3840px-Grey_heron_2022_03_18_01.jpg</t>
         </is>
       </c>
     </row>
@@ -2772,9 +2869,10 @@
           <t>Ground-feeding (terrestrial specialist)</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/7/79/Gallus_sonneratii_%28Bandipur%29%2C_crop.jpg</t>
         </is>
       </c>
     </row>
@@ -2819,9 +2917,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/3/33/Gebirgsstelze_im_Geo-Naturpark_Bergstra%C3%9Fe-Odenwald.jpg/3840px-Gebirgsstelze_im_Geo-Naturpark_Bergstra%C3%9Fe-Odenwald.jpg</t>
         </is>
       </c>
     </row>
@@ -2866,9 +2965,10 @@
           <t>Arboreal (low to midstory)</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/e/e7/Gray-bellied_Cuckoo_in_Bhigwan_August_2025_by_Tisha_Mukherjee_05.jpg/3840px-Gray-bellied_Cuckoo_in_Bhigwan_August_2025_by_Tisha_Mukherjee_05.jpg</t>
         </is>
       </c>
     </row>
@@ -2918,6 +3018,11 @@
           <t>Lantana-associated</t>
         </is>
       </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/0/03/Grey-breasted_prinia_%28Prinia_hodgsonii%29_by_Shantanu_Kuveskar.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2960,9 +3065,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/9/90/Treron_pompadora_affinis.JPG</t>
         </is>
       </c>
     </row>
@@ -3007,9 +3113,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/c/c8/Grey-headed_Bulbul.jpg</t>
         </is>
       </c>
     </row>
@@ -3059,6 +3166,11 @@
           <t>Lantana-associated</t>
         </is>
       </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/5/5c/Greater_coucal_crop.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3106,6 +3218,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/8/86/Chrysocolaptes_guttacristatus%2C_Kaeng_Krachan.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3153,6 +3270,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/9/91/GRTDrongo_Sandeep.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3195,9 +3317,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/9/92/Green-Sandpiper-Sandeep.jpg</t>
         </is>
       </c>
     </row>
@@ -3242,9 +3365,10 @@
           <t>Lower shrub layer / near-ground (low arboreal)</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/8/88/Green_warbler.jpg</t>
         </is>
       </c>
     </row>
@@ -3289,9 +3413,10 @@
           <t>Arboreal (midstory to canopy)</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/4/4e/Greenish_Warbler_Sikkim_India_11.05.2014.jpg</t>
         </is>
       </c>
     </row>
@@ -3336,9 +3461,10 @@
           <t>Ground-feeding (terrestrial)</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/0/05/Indian_Blackbird_at_Kotagiri.jpg/3840px-Indian_Blackbird_at_Kotagiri.jpg</t>
         </is>
       </c>
     </row>
@@ -3383,9 +3509,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/d/de/Larvivora_brunnea%2C_male%2C_Nandi_Hills.jpg</t>
         </is>
       </c>
     </row>
@@ -3430,9 +3557,10 @@
           <t>Arboreal (midstory to canopy)</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/5/51/IndianGoldenOriole_M.jpg</t>
         </is>
       </c>
     </row>
@@ -3477,9 +3605,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/5/5d/Indian_Grey_Hornbill_I_IMG_4051.jpg</t>
         </is>
       </c>
     </row>
@@ -3524,9 +3653,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/1/1f/Caprimulgus_asiaticus.jpg/3840px-Caprimulgus_asiaticus.jpg</t>
         </is>
       </c>
     </row>
@@ -3576,6 +3706,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/f/ff/Indian_paradise_flycatcher_%282018%29.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3618,9 +3753,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/7/7f/Peacock_on_tree_%2852077240794%29.jpg</t>
         </is>
       </c>
     </row>
@@ -3665,9 +3801,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/e/ef/Indian_pitta_%28Pitta_brachyura%29_Photograph_by_Shantanu_Kuveskar.jpg</t>
         </is>
       </c>
     </row>
@@ -3712,9 +3849,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/2/28/Indian_Robin_%28Copsychus_fulicatus%29%2C_Koottanad%2C_Palakkad_district%2C_Kerala_1.jpg</t>
         </is>
       </c>
     </row>
@@ -3759,9 +3897,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/0/06/Indian_roller_-_Timbi_Lake%2C_Vadodara_2023-12-03.jpg</t>
         </is>
       </c>
     </row>
@@ -3811,6 +3950,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/d/d6/IndianScimitarBabbler.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3853,9 +3997,10 @@
           <t>Arboreal</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/c/cc/Indian_white-eye_%28Zosterops_palpebrosus_egregius%29.jpg</t>
         </is>
       </c>
     </row>
@@ -3900,9 +4045,10 @@
           <t>Ground-feeding</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/9/90/Jerdon%27s_bushlark_%28Mirafra_affinis%29.jpg</t>
         </is>
       </c>
     </row>
@@ -3952,6 +4098,11 @@
           <t>Lantana-associated</t>
         </is>
       </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/4/48/Jungle_babbler_%28Turdoides_striata%29_Photograph_by_Shantanu_Kuveskar.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3994,9 +4145,10 @@
           <t>Ground-feeding + arboreal use (mixed)</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I76" t="inlineStr"/>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/c/c0/Jungle_Myna_%28Acridotheres_fuscus%29_on_Kapok_%28Ceiba_pentandra%29_in_Kolkata_I_IMG_1340.jpg</t>
         </is>
       </c>
     </row>
@@ -4041,9 +4193,10 @@
           <t>Arboreal (low to midstory perch hunter)</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I77" t="inlineStr"/>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/3/3c/Jungle_owlet_3.jpg</t>
         </is>
       </c>
     </row>
@@ -4093,6 +4246,11 @@
           <t>Lantana-associated</t>
         </is>
       </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/b/bb/Jungle_Prinia_in_Saswad_August_2025_by_Tisha_Mukherjee_02.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4135,9 +4293,10 @@
           <t>Mixed (arboreal + ground + aerial)</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I79" t="inlineStr"/>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/3/3a/Jungle_crow_%28Close-up_of_the_head_area%29%2C_Tenn%C5%8Dji_Park%2C_Osaka_II.jpg/3840px-Jungle_crow_%28Close-up_of_the_head_area%29%2C_Tenn%C5%8Dji_Park%2C_Osaka_II.jpg</t>
         </is>
       </c>
     </row>
@@ -4182,9 +4341,10 @@
           <t>Arboreal (lower to midstory)</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I80" t="inlineStr"/>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/d/dc/Large-billed_Leaf_Warbler_%28Phylloscopus_magnirostris%29.jpg</t>
         </is>
       </c>
     </row>
@@ -4229,9 +4389,10 @@
           <t>Ground-feeding (terrestrial)</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I81" t="inlineStr"/>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/0/05/140_Laughing_dove_in_Twyfelfontein_Photo_by_Giles_Laurent.jpg/3840px-140_Laughing_dove_in_Twyfelfontein_Photo_by_Giles_Laurent.jpg</t>
         </is>
       </c>
     </row>
@@ -4276,9 +4437,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I82" t="inlineStr"/>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/7/74/%D0%A1%D0%BB%D0%B0%D0%B2%D0%BA%D0%B0-%D0%B7%D0%B0%D0%B2%D0%B8%D1%80%D1%83%D1%88%D0%BA%D0%B0_%28Sylvia_curruca%29.jpg</t>
         </is>
       </c>
     </row>
@@ -4323,9 +4485,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I83" t="inlineStr"/>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/8/84/Little_grebe_Zwergtaucher.jpg</t>
         </is>
       </c>
     </row>
@@ -4370,9 +4533,10 @@
           <t>Arboreal (low to midstory)</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I84" t="inlineStr"/>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/a/aa/Loten%27sSunbird%28M%29.jpg</t>
         </is>
       </c>
     </row>
@@ -4417,9 +4581,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I85" t="inlineStr"/>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/1/11/Malabar_Barbet_%28Psilopogon_malabaricus%29_-_Male_-_Sakleshpur_-_India_-2009.jpg</t>
         </is>
       </c>
     </row>
@@ -4464,9 +4629,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I86" t="inlineStr"/>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/b/bd/Ocyceros_griseus_-India-6-4c.jpg</t>
         </is>
       </c>
     </row>
@@ -4516,6 +4682,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/5/5b/Malabar_or_Blue-winged_parakeet_%28Psittacula_columboides%29_by_Shantanu_Kuveskar.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4563,6 +4734,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/4/4c/Back_Whistling_Thrush_Sheikalmudi_Feb26_A7CR_10052.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4605,9 +4781,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I89" t="inlineStr"/>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/d/de/Blissful_Rare_Sighting_Malabar_Woodshrik_01%2C_crop.jpg</t>
         </is>
       </c>
     </row>
@@ -4657,6 +4834,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/1/1c/Dicaeum_concolor.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4704,6 +4886,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/9/99/Orange_Minivet%2C_Ganeshgudi%2C_28_FEB_2016%2C_Vimal_Rajyaguru.jpg/3840px-Orange_Minivet%2C_Ganeshgudi%2C_28_FEB_2016%2C_Vimal_Rajyaguru.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4751,6 +4938,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/1/13/Zoothera_citrina_-_Khao_Yai.jpg/3840px-Zoothera_citrina_-_Khao_Yai.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4793,9 +4985,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/2/2a/Oriental_magpie-robin_%28Copsychus_saularis_ceylonensis%29_male.jpg</t>
         </is>
       </c>
     </row>
@@ -4840,9 +5033,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/a/a0/Osprey_Perched_Snag_Heislerville.jpg</t>
         </is>
       </c>
     </row>
@@ -4887,9 +5081,10 @@
           <t>Arboreal (upper shrub to canopy)</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/9/9a/Pale_billed_Flowerpecker2.jpg</t>
         </is>
       </c>
     </row>
@@ -4934,9 +5129,10 @@
           <t>Arboreal (canopy to upper midstory)</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/d/d8/104_Male_Plum-headed_parakeet_eating_in_Jim_Corbett_National_Park_Photo_by_Giles_Laurent.jpg/3840px-104_Male_Plum-headed_parakeet_eating_in_Jim_Corbett_National_Park_Photo_by_Giles_Laurent.jpg</t>
         </is>
       </c>
     </row>
@@ -4986,6 +5182,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/5/59/Pellorneum_ruficeps_-_Khao_Yai.jpg/3840px-Pellorneum_ruficeps_-_Khao_Yai.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5028,9 +5229,10 @@
           <t>Arboreal (low to midstory)</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I98" t="inlineStr"/>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/7/7d/Purple_Sunbird_%28Nectarinia_asiatica%29-_Male_%28Breeding%29_on_Kapok_%28Ceiba_pentandra%29_in_Kolkata_I_IMG_1893.jpg</t>
         </is>
       </c>
     </row>
@@ -5075,9 +5277,10 @@
           <t>Arboreal</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I99" t="inlineStr"/>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/5/5a/PR-SunbirdM-Sandeep.jpg</t>
         </is>
       </c>
     </row>
@@ -5127,6 +5330,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/6/69/RED_SPURFOWL_NHOLE.png</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5169,9 +5377,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I101" t="inlineStr"/>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/e/eb/Red-rumped_swallow_in_Calpe%2C_Spain_-_May_2018_01.jpg</t>
         </is>
       </c>
     </row>
@@ -5221,6 +5430,11 @@
           <t>Lantana-associated</t>
         </is>
       </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/8/86/Red-vented_bulbul_-_Jamnagar_2023-11-13.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5263,9 +5477,10 @@
           <t>Ground-feeding</t>
         </is>
       </c>
-      <c r="I103" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I103" t="inlineStr"/>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/4/4e/Red-wattled_lapwing_%28Vanellus_indicus%29_Photograph_by_Shantanu_Kuveskar.jpg</t>
         </is>
       </c>
     </row>
@@ -5310,9 +5525,10 @@
           <t>Low to midstory arboreal</t>
         </is>
       </c>
-      <c r="I104" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I104" t="inlineStr"/>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/f/f7/Red-whiskered_bulbul_-_Pycnonotous_jocosus.png</t>
         </is>
       </c>
     </row>
@@ -5357,9 +5573,10 @@
           <t>Arboreal (midstory to canopy) + occasional ground use</t>
         </is>
       </c>
-      <c r="I105" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I105" t="inlineStr"/>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/7/7a/Rufous_treepie_%28Dendrocitta_vagabunda_vagabunda%29_Jahalana_pair.jpg</t>
         </is>
       </c>
     </row>
@@ -5404,9 +5621,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I106" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I106" t="inlineStr"/>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/8/83/Rufous_woodpecker.jpg</t>
         </is>
       </c>
     </row>
@@ -5451,9 +5669,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I107" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I107" t="inlineStr"/>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/f/fe/Shikra1.jpg</t>
         </is>
       </c>
     </row>
@@ -5503,6 +5722,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/4/40/Pericrocotus_cinnamomeus%2C_Small_minivet_%28male%29_-_Bangkok_%2825838143941%29.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -5545,9 +5769,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I109" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I109" t="inlineStr"/>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/9/9a/Starling_bird_%28India%2C_2012%29.jpg</t>
         </is>
       </c>
     </row>
@@ -5592,9 +5817,10 @@
           <t>Ground-feeding</t>
         </is>
       </c>
-      <c r="I110" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I110" t="inlineStr"/>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/6/6d/Spotted_dove_%28Spilopelia_chinensis_suratensis%29.jpg</t>
         </is>
       </c>
     </row>
@@ -5639,9 +5865,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I111" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I111" t="inlineStr"/>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/0/01/Stork-billed_Kingfisher_Baranagar_Kolkata_West_Bengal_India_21.04.2014.jpg</t>
         </is>
       </c>
     </row>
@@ -5686,9 +5913,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I112" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I112" t="inlineStr"/>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/4/4d/Syke%27s_Warbler_%28Hippolais_rama%29_on_Vilaiti_Siris_%28Samanea_saman%29_in_Kolkata_W_IMG_4659.jpg</t>
         </is>
       </c>
     </row>
@@ -5733,9 +5961,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I113" t="inlineStr"/>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/6/66/Taiga_Flycatcher.jpg</t>
         </is>
       </c>
     </row>
@@ -5780,9 +6009,10 @@
           <t>Lower shrub layer (low arboreal, near-ground)</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I114" t="inlineStr"/>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/b/bc/Tawny_bellied_warbler_2_by_David_Raju_%28cropped%29.jpg/3840px-Tawny_bellied_warbler_2_by_David_Raju_%28cropped%29.jpg</t>
         </is>
       </c>
     </row>
@@ -5827,9 +6057,10 @@
           <t>Arboreal</t>
         </is>
       </c>
-      <c r="I115" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I115" t="inlineStr"/>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/f/f0/Dicaeum_agile_modestum_-_Kaeng_Krachan.jpg</t>
         </is>
       </c>
     </row>
@@ -5879,6 +6110,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/8/8e/Tickell%27s_blue_flycatcher_%28Cyornis_tickelliae%29_Photograph_By_Shantanu_Kuveskar.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -5921,9 +6157,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I117" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I117" t="inlineStr"/>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/6/6d/Tree_pipit_-_Jamnagar_2021-10-16.jpg</t>
         </is>
       </c>
     </row>
@@ -5973,6 +6210,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/c/c6/Velvet-fronted_Nuthatch_%E0%A4%AE%E0%A4%96%E0%A4%AE%E0%A4%B2%E0%A5%80_%E0%A4%AE%E0%A4%9F%E0%A5%8D%E0%A4%9F%E0%A4%BE.jpg/3840px-Velvet-fronted_Nuthatch_%E0%A4%AE%E0%A4%96%E0%A4%AE%E0%A4%B2%E0%A5%80_%E0%A4%AE%E0%A4%9F%E0%A5%8D%E0%A4%9F%E0%A4%BE.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6015,9 +6257,10 @@
           <t>Arboreal (midstory to open perch level)</t>
         </is>
       </c>
-      <c r="I119" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I119" t="inlineStr"/>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/5/56/%E0%A6%85%E0%A6%AE%E0%A7%8D%E0%A6%AC%E0%A6%B0_%E0%A6%9A%E0%A7%81%E0%A6%9F%E0%A6%95%E0%A6%BF_-_Verditer_flycatcher_%28Eumyias_thalassinus%29%2C_Naogaon%2C_Bangladesh.jpg</t>
         </is>
       </c>
     </row>
@@ -6062,9 +6305,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I120" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I120" t="inlineStr"/>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/0/0d/Loriculus_vernalis_-Ganeshgudi%2C_Karnataka%2C_India_-male-8-1c.jpg</t>
         </is>
       </c>
     </row>
@@ -6109,9 +6353,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I121" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I121" t="inlineStr"/>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/a/a1/White-bellied_treepie_-_Dendrocitta_leucogastra%29.jpg/3840px-White-bellied_treepie_-_Dendrocitta_leucogastra%29.jpg</t>
         </is>
       </c>
     </row>
@@ -6156,9 +6401,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I122" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I122" t="inlineStr"/>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/0/0f/Amaurornis_phoenicurus_-_Singapore_Botanic_Gardens.jpg</t>
         </is>
       </c>
     </row>
@@ -6208,6 +6454,11 @@
           <t>Lantana-associated</t>
         </is>
       </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/d/db/White_browed_bulbul-4E_%28cropped%29.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -6255,6 +6506,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/thumb/5/5f/White-cheeked_barbet_Christ_University_-_Birdwalk_%282%29.jpg/3840px-White-cheeked_barbet_Christ_University_-_Birdwalk_%282%29.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -6297,9 +6553,10 @@
           <t>Perch hunter (arboreal + ground/water strike)</t>
         </is>
       </c>
-      <c r="I125" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I125" t="inlineStr"/>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/c/c8/White-throated_kingfisher_%28Halcyon_smyrnensis%29_Galle.jpg</t>
         </is>
       </c>
     </row>
@@ -6349,6 +6606,11 @@
           <t>Lantana-associated</t>
         </is>
       </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/0/0e/Yellow-billed_babbler_%28Argya_affinis_taprobanus%29.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -6396,6 +6658,11 @@
           <t>Recovery-associated</t>
         </is>
       </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/a/ac/Yellow-browed_bulbul.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -6438,9 +6705,10 @@
           <t>Primarily ground-feeding</t>
         </is>
       </c>
-      <c r="I128" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I128" t="inlineStr"/>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/d/da/Yellow-eyed_babbler_%28Chrysomma_sinense%29_Photograph_by_Shantanu_Kuveskar.jpg</t>
         </is>
       </c>
     </row>
@@ -6485,9 +6753,10 @@
           <t>Ground + low arboreal</t>
         </is>
       </c>
-      <c r="I129" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I129" t="inlineStr"/>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/0/00/Petronia_xanthocollis_-Haryana%2C_India_-male-8.jpg</t>
         </is>
       </c>
     </row>
@@ -6532,9 +6801,10 @@
           <t>Primarily arboreal</t>
         </is>
       </c>
-      <c r="I130" t="inlineStr">
-        <is>
-          <t>None</t>
+      <c r="I130" t="inlineStr"/>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>https://upload.wikimedia.org/wikipedia/commons/3/31/Zitting_cisticola_2024_04_19_%28cropped%29.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>